<commit_message>
Site: one CTA wording everywhere («Prøv gratis», «Prøv gratis i 15 dager»), digits in the shared anonymity and start texts; /priser sheet fixture follows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U8NqjgPf4GAveNTnTAzZjT
</commit_message>
<xml_diff>
--- a/tests/unit/fixtures/site-sheet-openpyxl.xlsx
+++ b/tests/unit/fixtures/site-sheet-openpyxl.xlsx
@@ -755,12 +755,12 @@
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>Start gratis</t>
+          <t>Prøv gratis</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>Start free</t>
+          <t>Try it free</t>
         </is>
       </c>
       <c r="E18" s="1" t="inlineStr"/>
@@ -773,12 +773,12 @@
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>Ingen avdeling vises før minst fem har svart.</t>
+          <t>Ingen avdeling vises før minst 5 har svart.</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>No department is shown until at least five have answered.</t>
+          <t>No department is shown until at least 5 have answered.</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr"/>
@@ -935,12 +935,12 @@
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>Start gratis</t>
+          <t>Prøv gratis</t>
         </is>
       </c>
       <c r="D28" s="1" t="inlineStr">
         <is>
-          <t>Start free</t>
+          <t>Try it free</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr"/>
@@ -1115,12 +1115,12 @@
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t>Start gratis</t>
+          <t>Prøv gratis</t>
         </is>
       </c>
       <c r="D38" s="1" t="inlineStr">
         <is>
-          <t>Start free</t>
+          <t>Try it free</t>
         </is>
       </c>
       <c r="E38" s="1" t="inlineStr"/>
@@ -1449,12 +1449,12 @@
       </c>
       <c r="C57" s="1" t="inlineStr">
         <is>
-          <t>Skriv inn organisasjonsnummeret, så henter vi resten fra Brønnøysundregistrene. Dere er i gang på tre minutter, og trenger ikke oppgi kort før dere har bestemt dere.</t>
+          <t>Skriv inn organisasjonsnummeret, så henter vi resten fra Brønnøysundregistrene. Dere er i gang på 3 minutter, og trenger ikke oppgi kort før dere har bestemt dere.</t>
         </is>
       </c>
       <c r="D57" s="1" t="inlineStr">
         <is>
-          <t>Enter the organisation number and we fetch the rest from the Norwegian company register. You are up and running in three minutes, and do not need to give card details before you have decided.</t>
+          <t>Enter the organisation number and we fetch the rest from the Norwegian company register. You are up and running in 3 minutes, and do not need to give card details before you have decided.</t>
         </is>
       </c>
       <c r="E57" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Public site: 5 is the default anonymity limit, not a fixed one (D-199)
The floor becomes 3; every organisation starts at 5, the daglig leder can
lower it to 3 or 4 for a small team, it can be raised to 10, and a round
keeps the limit it opened with. The site, the landing pages, the articles,
the industry pages, /sikkerhet and /vilkar § 6 said the limit was 5 and
could not be lowered. They now say 5 by default, strongly recommended, and
never below 3, with the trade-off (fewer answers, easier to recognise who
said what) stated once where a page explains why.

47 keys per language in seo.* and site.*, the five industry pages (no) and
two English ones, the share cards regenerated for the new pill, and the
/priser sheet fixture following its three changed texts. /vilkar stays
Versjon 1 from 2 October 2026; the draft's status block notes the change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U8NqjgPf4GAveNTnTAzZjT
</commit_message>
<xml_diff>
--- a/tests/unit/fixtures/site-sheet-openpyxl.xlsx
+++ b/tests/unit/fixtures/site-sheet-openpyxl.xlsx
@@ -539,12 +539,12 @@
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>Da får dere tall for hele virksomheten. En avdeling vises bare når minst 5 i den har svart. Er færre enn 5 med på å svare, vises ingen tall – da kunne ikke svarene vært anonyme.</t>
+          <t>Da får dere tall for hele virksomheten. Som standard vises en avdeling når minst 5 i den har svart; færre teller med i helheten. For små team kan daglig leder senke grensen til 3, men 5 er sterkt anbefalt – jo færre svar, jo lettere er det å kjenne igjen hvem som sa hva.</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>Then you get figures for the whole organisation. A department is shown only once at least 5 people in it have answered. If fewer than 5 answer, no figures are shown – the answers could not be anonymous then.</t>
+          <t>Then you get figures for the whole organisation. By default a department is shown once at least 5 people in it have answered; fewer count in the whole. For small teams the managing director can lower the limit to 3, but 5 is strongly recommended – the fewer the answers, the easier it is to recognise who said what.</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr"/>
@@ -575,12 +575,12 @@
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>Ja. Vi lagrer aldri navn, e-postadresse eller IP-adresse sammen med svaret – det finnes ingen kolonne som kunne holdt koblingen. Og ingen gruppe vises før minst 5 personer har svart.</t>
+          <t>Ja. Vi lagrer aldri navn, e-postadresse eller IP-adresse sammen med svaret – det finnes ingen kolonne som kunne holdt koblingen. Og som standard vises ingen gruppe før minst 5 personer har svart; grensen kan aldri settes under 3.</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>Yes. We never store a name, e-mail address or IP address with the answer – there is no column that could hold the link. And no group is shown until at least 5 people have answered.</t>
+          <t>Yes. We never store a name, e-mail address or IP address with the answer – there is no column that could hold the link. And by default no group is shown until at least 5 people have answered; the limit can never be set below 3.</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr"/>
@@ -773,12 +773,12 @@
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>Ingen avdeling vises før minst 5 har svart.</t>
+          <t>Som standard vises ingen avdeling før minst 5 har svart.</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>No department is shown until at least 5 have answered.</t>
+          <t>By default, no department is shown until at least 5 have answered.</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
«Arbeidsmiljøundersøkelse» leads the titles; free on the home page in SEO too (D-227)
Neither «medarbeiderundersøkelse» nor «arbeidsmiljøundersøkelse» is the
law's word, and Arbeidstilsynet uses both (sources in
docs/marketing/terminologi-arbeidsmiljoundersokelse.md). «Arbeidsmiljø-
undersøkelse» matches the duty the product documents, so it now leads the
home description, the five industry titles, Pris, Plattform, Bruksområder,
the articles index and the Bransjer H1. «Medarbeiderundersøkelse» stays in
the home title and on the pages that rank for it; «arbeidsmiljøkartlegging»
leaves the titles. The home description and Pris say free to start. Page map
and the sheet fixture follow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U8NqjgPf4GAveNTnTAzZjT
</commit_message>
<xml_diff>
--- a/tests/unit/fixtures/site-sheet-openpyxl.xlsx
+++ b/tests/unit/fixtures/site-sheet-openpyxl.xlsx
@@ -466,12 +466,12 @@
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>Priser: gratis å starte, fra 265 kr/mnd | Orgpuls</t>
+          <t>Priser: gratis arbeidsmiljøundersøkelse | Orgpuls</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Pricing: free to start, from NOK 265/month | Orgpuls</t>
+          <t>Pricing: free work environment survey | Orgpuls</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr"/>
@@ -484,12 +484,12 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>Gratis for hovedkartleggingen. Liten 265 kr og Vanlig 565 kr i måneden eks. mva., to måneder gratis med årlig avtale. 15 dager med alt, uten kort.</t>
+          <t>Gratis årlig arbeidsmiljøundersøkelse. Liten 265 kr og Vanlig 565 kr i måneden eks. mva., to måneder gratis med årlig avtale. 15 dager med alt, uten kort.</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>Free for the main survey. Small NOK 265 and Usual NOK 565 a month excl. VAT, two months free with a yearly agreement. 15 days with everything, no card. (corrected)
+          <t>Free yearly work environment survey. Small NOK 265 and Usual NOK 565 a month excl. VAT, two months free yearly. 15 days with everything, no card. (corrected)
 second line</t>
         </is>
       </c>
@@ -665,12 +665,12 @@
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>Medarbeiderundersøkelse som kartlegger det psykososiale arbeidsmiljøet, gjør funnene om til tiltak og viser om de virker. 15 dager gratis.</t>
+          <t>Arbeidsmiljøundersøkelse for kartleggingen arbeidsmiljøloven krever: anonymt, med tiltak og rapport til Arbeidstilsynet. Gratis å starte.</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>An employee survey that maps the psychosocial working environment, turns the findings into measures and shows whether they work. 15 days free.</t>
+          <t>A work environment survey for the mapping Norwegian law requires: anonymous, with measures and a report for the Labour Inspection Authority. Free to start.</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr"/>

</xml_diff>